<commit_message>
added Extent Reports TestListener and Excel collection
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/srikanthkunnkunuru/api-framework/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96C2FFF6-E697-234E-9069-8E8DFB62B68E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F0FD863-E2D6-2F48-B42E-E94AFB1F2686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="740" windowWidth="28040" windowHeight="16680" xr2:uid="{0F83192F-9B1B-8D45-AFFE-1993D8ACAB45}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" activeTab="1" xr2:uid="{0F83192F-9B1B-8D45-AFFE-1993D8ACAB45}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="ApiCollection" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,51 +36,42 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>job</t>
-  </si>
-  <si>
-    <t>srikanth</t>
-  </si>
-  <si>
-    <t>varsha</t>
-  </si>
-  <si>
-    <t>jai</t>
-  </si>
-  <si>
-    <t>neetika</t>
-  </si>
-  <si>
-    <t>anoushka</t>
-  </si>
-  <si>
-    <t>arushi</t>
-  </si>
-  <si>
-    <t>QA</t>
-  </si>
-  <si>
-    <t>SALES</t>
-  </si>
-  <si>
-    <t>DEVLOPER</t>
-  </si>
-  <si>
-    <t>HR</t>
-  </si>
-  <si>
-    <t>MARKETING</t>
-  </si>
-  <si>
-    <t>mahesh</t>
-  </si>
-  <si>
-    <t>sales</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="12">
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>paylod</t>
+  </si>
+  <si>
+    <t>expectd status</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>PUT</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>/users</t>
+  </si>
+  <si>
+    <t>/users/2</t>
+  </si>
+  <si>
+    <t>{"name":"Srikanth","job":"QA"}</t>
+  </si>
+  <si>
+    <t>{"name":"Updated","job":"Senior QA"}</t>
   </si>
 </sst>
 </file>
@@ -431,71 +423,151 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D07FAE31-BFC4-A24F-96A1-607D46768418}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="31.6640625" customWidth="1"/>
+    <col min="2" max="2" width="61.6640625" customWidth="1"/>
+    <col min="3" max="3" width="62.6640625" customWidth="1"/>
+    <col min="4" max="4" width="45.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>204</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35C32FCD-C400-2340-ADB1-5540EF62F7FB}">
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>